<commit_message>
Cosmetici 09/2026: revisão sistemática com todos os relatórios da pasta
- Registro de Saídas do ERP x XML nota a nota (UF, CFOP, valores, ICMS,
  ST, IPI) - leitor do PDF do Cosmos e cruzamento automático
- mesmo produto com NCM/IPI diferentes; PIS/COFINS informado no XML das
  industrializações x apuração
- checklist refeito: matriz NCM x CFOP x CST das saídas e entradas,
  extrato x documentos (boletos da Remazzo, TEX Courier), NFS-e, CT-e

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Apuracao_Fiscal_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Apuracao_Fiscal_Cosmetici_09-2026.xlsx
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="B67" s="13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68">
@@ -1311,7 +1311,7 @@
         </is>
       </c>
       <c r="B68" s="11" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="69">
@@ -1609,7 +1609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1934,116 +1934,116 @@
       <c r="G13" s="16" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Saídas</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>NCM x PIS/COFINS monofásico</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>Nenhuma ocorrência</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>Lei 10.147/2000</t>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Mesmo produto com NCM/IPI diferentes no mês</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>1 MÉDIA (aba Divergências)</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>VERIFICAR</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>TIPI (Decreto 11.158/2022); RIPI art. 189</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr"/>
       <c r="G14" s="16" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>Entradas</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>Fornecedor sem histórico (insumo x uso e consumo)</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>11 MÉDIA (aba Divergências)</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>VERIFICAR</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>LC 87/96 art. 20 e 33, I</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Saídas</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>PIS/COFINS informado no XML x apuração</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>1 BAIXA (aba Divergências)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>INFORMATIVO</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>Lei 10.147/2000; Lei 11.051/2004 art. 10</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr"/>
       <c r="G15" s="16" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Entradas</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Notas desconhecidas/manifestadas</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Nenhuma ocorrência</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>Ajuste SINIEF 07/05</t>
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Saídas</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>XML x Registro de Saídas do ERP (nota a nota: UF, CFOP, valores, ICMS, IPI, ST)</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>2 ALTA, 1 BAIXA (aba Divergências)</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>VERIFICAR</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>Ajuste SINIEF 02/09 (EFD)</t>
         </is>
       </c>
       <c r="F16" s="16" t="inlineStr"/>
       <c r="G16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Entradas</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>Remessas recebidas sem retorno (estoque de terceiros)</t>
-        </is>
-      </c>
-      <c r="C17" s="20" t="inlineStr">
-        <is>
-          <t>12 BAIXA (aba Divergências)</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>INFORMATIVO</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>RICMS/PR (industrialização por encomenda)</t>
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Saídas</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>NCM x PIS/COFINS monofásico</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Nenhuma ocorrência</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>Lei 10.147/2000</t>
         </is>
       </c>
       <c r="F17" s="16" t="inlineStr"/>
@@ -2052,17 +2052,17 @@
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>CT-e</t>
+          <t>Entradas</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Crédito do frete segue a natureza da NF-e transportada</t>
+          <t>Fornecedor sem histórico (insumo x uso e consumo)</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>1 MÉDIA (aba Divergências)</t>
+          <t>11 MÉDIA (aba Divergências)</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
@@ -2079,62 +2079,149 @@
       <c r="G18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t>Serviços</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>NFS-e tomadas: retenção de IRRF e PIS/COFINS/CSLL</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>1 MÉDIA, 1 BAIXA (aba Divergências)</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>VERIFICAR</t>
-        </is>
-      </c>
-      <c r="E19" s="19" t="inlineStr">
-        <is>
-          <t>Lei 10.833/2003 art. 30 e 31 §3º (dispensa até R$ 10); RIR/2018 art. 714 e 716; IN SRF 459/2004</t>
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Entradas</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Notas desconhecidas/manifestadas</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Nenhuma ocorrência</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Ajuste SINIEF 07/05</t>
         </is>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="16" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>SPED</t>
-        </is>
-      </c>
-      <c r="B20" s="21" t="inlineStr">
-        <is>
-          <t>XML x SPED (notas faltando de um lado ou do outro)</t>
-        </is>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>SPED do mês ainda não existe</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>NÃO EXECUTADO</t>
-        </is>
-      </c>
-      <c r="E20" s="21" t="inlineStr">
-        <is>
-          <t>Guia Prático EFD ICMS/IPI</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Entradas</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Remessas recebidas sem retorno (estoque de terceiros)</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>12 BAIXA (aba Divergências)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>INFORMATIVO</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>RICMS/PR (industrialização por encomenda)</t>
         </is>
       </c>
       <c r="F20" s="16" t="inlineStr"/>
       <c r="G20" s="16" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>CT-e</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Crédito do frete segue a natureza da NF-e transportada</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>1 MÉDIA (aba Divergências)</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>VERIFICAR</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>LC 87/96 art. 20 e 33, I</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr"/>
+      <c r="G21" s="16" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>NFS-e tomadas: retenção de IRRF e PIS/COFINS/CSLL</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>1 MÉDIA, 1 BAIXA (aba Divergências)</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>VERIFICAR</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>Lei 10.833/2003 art. 30 e 31 §3º (dispensa até R$ 10); RIR/2018 art. 714 e 716; IN SRF 459/2004</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr"/>
+      <c r="G22" s="16" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>SPED</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>XML x SPED (notas faltando de um lado ou do outro)</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>SPED do mês ainda não existe</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>NÃO EXECUTADO</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>Guia Prático EFD ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr"/>
+      <c r="G23" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -33064,7 +33151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -33315,56 +33402,52 @@
       <c r="G11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>CFOP revenda x produção</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>NF 8967/1 11/09 GULA COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>1 item(ns) com CFOP 6102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="n">
-        <v>370.33</v>
-      </c>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>XML x Registro ERP</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>NF 8966/1 10/09 GULA COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>UF no XML SP x ERP PR</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="n"/>
       <c r="F12" s="16" t="inlineStr"/>
       <c r="G12" s="16" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>CFOP revenda x produção</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>NF 8969/1 14/09 GULA COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>2 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="n">
-        <v>811.99</v>
-      </c>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>XML x Registro ERP</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>NF 8967/1 11/09 GULA COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>UF no XML SP x ERP PR</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="n"/>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="16" t="inlineStr"/>
     </row>
@@ -33381,16 +33464,16 @@
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>NF 8978/1 16/09 GULA COSMETICOS LTDA</t>
+          <t>NF 8967/1 11/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>9 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>1 item(ns) com CFOP 6102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
-        <v>1698.59</v>
+        <v>370.33</v>
       </c>
       <c r="F14" s="16" t="inlineStr"/>
       <c r="G14" s="16" t="inlineStr"/>
@@ -33408,16 +33491,16 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>NF 8980/1 17/09 GULA COSMETICOS LTDA</t>
+          <t>NF 8969/1 14/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>19 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>2 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E15" s="23" t="n">
-        <v>11620.79</v>
+        <v>811.99</v>
       </c>
       <c r="F15" s="16" t="inlineStr"/>
       <c r="G15" s="16" t="inlineStr"/>
@@ -33435,16 +33518,16 @@
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>NF 8981/1 17/09 GULA COSMETICOS LTDA</t>
+          <t>NF 8978/1 16/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>9 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E16" s="23" t="n">
-        <v>1691.57</v>
+        <v>1698.59</v>
       </c>
       <c r="F16" s="16" t="inlineStr"/>
       <c r="G16" s="16" t="inlineStr"/>
@@ -33462,16 +33545,16 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>NF 8982/1 18/09 GULA COSMETICOS LTDA</t>
+          <t>NF 8980/1 17/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>19 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E17" s="23" t="n">
-        <v>6901.45</v>
+        <v>11620.79</v>
       </c>
       <c r="F17" s="16" t="inlineStr"/>
       <c r="G17" s="16" t="inlineStr"/>
@@ -33489,16 +33572,16 @@
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>NF 9003/1 23/09 GULA COSMETICOS LTDA</t>
+          <t>NF 8981/1 17/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>4 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E18" s="23" t="n">
-        <v>156.77</v>
+        <v>1691.57</v>
       </c>
       <c r="F18" s="16" t="inlineStr"/>
       <c r="G18" s="16" t="inlineStr"/>
@@ -33516,7 +33599,7 @@
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>NF 9006/1 23/09 GULA COSMETICOS LTDA</t>
+          <t>NF 8982/1 18/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -33525,7 +33608,7 @@
         </is>
       </c>
       <c r="E19" s="23" t="n">
-        <v>302.73</v>
+        <v>6901.45</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="16" t="inlineStr"/>
@@ -33543,16 +33626,16 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>NF 9009/1 23/09 GULA COSMETICOS LTDA</t>
+          <t>NF 9003/1 23/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>5 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>4 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E20" s="23" t="n">
-        <v>1529.47</v>
+        <v>156.77</v>
       </c>
       <c r="F20" s="16" t="inlineStr"/>
       <c r="G20" s="16" t="inlineStr"/>
@@ -33570,16 +33653,16 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>NF 9013/1 28/09 GULA COSMETICOS LTDA</t>
+          <t>NF 9006/1 23/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>2 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E21" s="23" t="n">
-        <v>618.45</v>
+        <v>302.73</v>
       </c>
       <c r="F21" s="16" t="inlineStr"/>
       <c r="G21" s="16" t="inlineStr"/>
@@ -33597,16 +33680,16 @@
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>NF 9014/1 28/09 GULA COSMETICOS LTDA</t>
+          <t>NF 9009/1 23/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>5 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E22" s="23" t="n">
-        <v>148.13</v>
+        <v>1529.47</v>
       </c>
       <c r="F22" s="16" t="inlineStr"/>
       <c r="G22" s="16" t="inlineStr"/>
@@ -33624,16 +33707,16 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>NF 9018/1 29/09 GULA COSMETICOS LTDA</t>
+          <t>NF 9013/1 28/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>2 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E23" s="23" t="n">
-        <v>139.49</v>
+        <v>618.45</v>
       </c>
       <c r="F23" s="16" t="inlineStr"/>
       <c r="G23" s="16" t="inlineStr"/>
@@ -33651,16 +33734,16 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>NF 9019/1 29/09 GULA COSMETICOS LTDA</t>
+          <t>NF 9014/1 28/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>41 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
+          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E24" s="23" t="n">
-        <v>6020.39</v>
+        <v>148.13</v>
       </c>
       <c r="F24" s="16" t="inlineStr"/>
       <c r="G24" s="16" t="inlineStr"/>
@@ -33673,21 +33756,21 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>CT-e sem crédito</t>
+          <t>CFOP revenda x produção</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>CT-e 5597996 CAXIAS DO SUL - EXPRESSO SAO MIGUEL S/A</t>
+          <t>NF 9018/1 29/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Frete de compra de outras: sem crédito - o crédito do frete segue a mercadoria (uso e consumo/outras não creditam - LC 87/96 art. 33, I). ICMS R$ 36.18 não aproveitado</t>
+          <t>1 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E25" s="23" t="n">
-        <v>36.18</v>
+        <v>139.49</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="16" t="inlineStr"/>
@@ -33700,21 +33783,21 @@
       </c>
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>Diferimento 5124</t>
+          <t>CFOP revenda x produção</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
+          <t>NF 9019/1 29/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>5124 para PR com CST 00 (ICMS R$ 108.44) enquanto 35 itens 5124 do mês saíram com diferimento (CST 51). Conferir se o diferimento se aplica a este cliente</t>
+          <t>41 item(ns) com CFOP 5102 (mercadoria de terceiros) e IPI destacado - produto fabricado pela COSMETICI sai com 5101/6101 (ou 5401 com ST). Conferir CFOP e natureza "VENDA DE MERCADORIAS"</t>
         </is>
       </c>
       <c r="E26" s="23" t="n">
-        <v>108.44</v>
+        <v>6020.39</v>
       </c>
       <c r="F26" s="16" t="inlineStr"/>
       <c r="G26" s="16" t="inlineStr"/>
@@ -33727,20 +33810,22 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Fornecedor sem histórico</t>
+          <t>CT-e sem crédito</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>ALTEC IND.COM.IMP.E EXP.LTDA. (67598292000187)</t>
+          <t>CT-e 5597996 CAXIAS DO SUL - EXPRESSO SAO MIGUEL S/A</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Natureza definida pelo NCM (sem histórico no SPED) - confirmar insumo (1101/2101) x uso e consumo (1556/2556)</t>
-        </is>
-      </c>
-      <c r="E27" s="23" t="n"/>
+          <t>Frete de compra de outras: sem crédito - o crédito do frete segue a mercadoria (uso e consumo/outras não creditam - LC 87/96 art. 33, I). ICMS R$ 36.18 não aproveitado</t>
+        </is>
+      </c>
+      <c r="E27" s="23" t="n">
+        <v>36.18</v>
+      </c>
       <c r="F27" s="16" t="inlineStr"/>
       <c r="G27" s="16" t="inlineStr"/>
     </row>
@@ -33752,20 +33837,22 @@
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>Fornecedor sem histórico</t>
+          <t>Diferimento 5124</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>BISPHARMA EMBALAGENS LTDA (59610485000188)</t>
+          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Natureza definida pelo NCM (sem histórico no SPED) - confirmar insumo (1101/2101) x uso e consumo (1556/2556)</t>
-        </is>
-      </c>
-      <c r="E28" s="23" t="n"/>
+          <t>5124 para PR com CST 00 (ICMS R$ 108.44) enquanto 35 itens 5124 do mês saíram com diferimento (CST 51). Conferir se o diferimento se aplica a este cliente</t>
+        </is>
+      </c>
+      <c r="E28" s="23" t="n">
+        <v>108.44</v>
+      </c>
       <c r="F28" s="16" t="inlineStr"/>
       <c r="G28" s="16" t="inlineStr"/>
     </row>
@@ -33782,7 +33869,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>CHEMYUNION LTDA (58309709000820)</t>
+          <t>ALTEC IND.COM.IMP.E EXP.LTDA. (67598292000187)</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -33807,7 +33894,7 @@
       </c>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA INDUSTRIAL PARANAENSE LTDA (04993269000177)</t>
+          <t>BISPHARMA EMBALAGENS LTDA (59610485000188)</t>
         </is>
       </c>
       <c r="D30" s="19" t="inlineStr">
@@ -33832,7 +33919,7 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>ELLOLIMP COMERCIO DE PRODUTOS DE HIGIENE E LIMPEZA LTDA (49547438000183)</t>
+          <t>CHEMYUNION LTDA (58309709000820)</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -33857,7 +33944,7 @@
       </c>
       <c r="C32" s="18" t="inlineStr">
         <is>
-          <t>HS INKLASER LTDA (18858535000163)</t>
+          <t>DISTRIBUIDORA INDUSTRIAL PARANAENSE LTDA (04993269000177)</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
@@ -33882,7 +33969,7 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>Lunaflexo Tecnologia Adesiva Eireli (06015875000143)</t>
+          <t>ELLOLIMP COMERCIO DE PRODUTOS DE HIGIENE E LIMPEZA LTDA (49547438000183)</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -33907,7 +33994,7 @@
       </c>
       <c r="C34" s="18" t="inlineStr">
         <is>
-          <t>MCASSAB COMERCIO E INDUSTRIA LTDA (49698723003110)</t>
+          <t>HS INKLASER LTDA (18858535000163)</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
@@ -33932,7 +34019,7 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>NewProv - Produtos para Laboratório Ltda (73636391000109)</t>
+          <t>Lunaflexo Tecnologia Adesiva Eireli (06015875000143)</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -33957,7 +34044,7 @@
       </c>
       <c r="C36" s="18" t="inlineStr">
         <is>
-          <t>PROVITAL DO BRASIL COM. DE INSUMOS PARA COSMETICOS LTDA (11340087000162)</t>
+          <t>MCASSAB COMERCIO E INDUSTRIA LTDA (49698723003110)</t>
         </is>
       </c>
       <c r="D36" s="19" t="inlineStr">
@@ -33982,7 +34069,7 @@
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>SCENTEC ESSENCIAS E FRAGRANCIAS LTDA (62514971000107)</t>
+          <t>NewProv - Produtos para Laboratório Ltda (73636391000109)</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -34002,22 +34089,20 @@
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Industrialização sem insumo</t>
+          <t>Fornecedor sem histórico</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
         <is>
-          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
+          <t>PROVITAL DO BRASIL COM. DE INSUMOS PARA COSMETICOS LTDA (11340087000162)</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>CFOP 5124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês. Confirmar o insumo enviado pelo encomendante; se não houve, é venda (5101/6101): PIS/COFINS monofásico 2,2%/10,3% em vez de 0,65%/3% (diferença ~R$ 39.61) e IPI tributado</t>
-        </is>
-      </c>
-      <c r="E38" s="23" t="n">
-        <v>556.05</v>
-      </c>
+          <t>Natureza definida pelo NCM (sem histórico no SPED) - confirmar insumo (1101/2101) x uso e consumo (1556/2556)</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="n"/>
       <c r="F38" s="16" t="inlineStr"/>
       <c r="G38" s="16" t="inlineStr"/>
     </row>
@@ -34029,22 +34114,20 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Industrialização sem insumo</t>
+          <t>Fornecedor sem histórico</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>NF 8979/1 17/09 BARBARA KAROLAINY DE SOUZA SILVA</t>
+          <t>SCENTEC ESSENCIAS E FRAGRANCIAS LTDA (62514971000107)</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>CFOP 6124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês. Confirmar o insumo enviado pelo encomendante; se não houve, é venda (5101/6101): PIS/COFINS monofásico 2,2%/10,3% em vez de 0,65%/3% (diferença ~R$ 337.29) e IPI tributado</t>
-        </is>
-      </c>
-      <c r="E39" s="23" t="n">
-        <v>4098</v>
-      </c>
+          <t>Natureza definida pelo NCM (sem histórico no SPED) - confirmar insumo (1101/2101) x uso e consumo (1556/2556)</t>
+        </is>
+      </c>
+      <c r="E39" s="23" t="n"/>
       <c r="F39" s="16" t="inlineStr"/>
       <c r="G39" s="16" t="inlineStr"/>
     </row>
@@ -34056,93 +34139,101 @@
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>NFS-e retenções</t>
+          <t>Industrialização sem insumo</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>NFS-e 18 01/09/2026 GENESIS ALIANCA</t>
+          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
         </is>
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>Serviço 0401 (medicina) de R$ 728.14, prestador fora do Simples: reter IRRF 1.5% R$ 10.92 + PIS/COFINS/CSLL 4,65% R$ 33.86 = R$ 44.78; descontado na nota R$ 10.92 (diferença R$ 33.86). Conferir pagamento e DARF 1708/5952</t>
+          <t>CFOP 5124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês. Confirmar o insumo enviado pelo encomendante; se não houve, é venda (5101/6101): PIS/COFINS monofásico 2,2%/10,3% em vez de 0,65%/3% (diferença ~R$ 39.61) e IPI tributado</t>
         </is>
       </c>
       <c r="E40" s="23" t="n">
-        <v>33.86</v>
+        <v>556.05</v>
       </c>
       <c r="F40" s="16" t="inlineStr"/>
       <c r="G40" s="16" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>BAIXA</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Carta de correção</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>NF 786/1 02/09 YAHWEH PRINT BRASIL LTDA</t>
-        </is>
-      </c>
-      <c r="D41" s="20" t="inlineStr">
-        <is>
-          <t>VOLUMES: 4 CAIXAS</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="n"/>
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>Industrialização sem insumo</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>NF 8979/1 17/09 BARBARA KAROLAINY DE SOUZA SILVA</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>CFOP 6124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês. Confirmar o insumo enviado pelo encomendante; se não houve, é venda (5101/6101): PIS/COFINS monofásico 2,2%/10,3% em vez de 0,65%/3% (diferença ~R$ 337.29) e IPI tributado</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="n">
+        <v>4098</v>
+      </c>
       <c r="F41" s="16" t="inlineStr"/>
       <c r="G41" s="16" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>BAIXA</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Carta de correção</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>NF 786/1 02/09 YAHWEH PRINT BRASIL LTDA</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="inlineStr"/>
-      <c r="E42" s="6" t="n"/>
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>NFS-e retenções</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>NFS-e 18 01/09/2026 GENESIS ALIANCA</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>Serviço 0401 (medicina) de R$ 728.14, prestador fora do Simples: reter IRRF 1.5% R$ 10.92 + PIS/COFINS/CSLL 4,65% R$ 33.86 = R$ 44.78; descontado na nota R$ 10.92 (diferença R$ 33.86). Conferir pagamento e DARF 1708/5952</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="n">
+        <v>33.86</v>
+      </c>
       <c r="F42" s="16" t="inlineStr"/>
       <c r="G42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>BAIXA</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Carta de correção</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>NF 8992/1 21/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D43" s="20" t="inlineStr">
-        <is>
-          <t>INDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NAS NFs 55874 de 21-09-2026</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="n"/>
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>Produto com tratamento diferente</t>
+        </is>
+      </c>
+      <c r="C43" s="18" t="inlineStr">
+        <is>
+          <t>NEUTRALIZANTE ALL NATURE - 500ML (cód. 51)</t>
+        </is>
+      </c>
+      <c r="D43" s="19" t="inlineStr">
+        <is>
+          <t>Mesmo produto vendido no mês com NCM/IPI diferentes: NCM 33059000 IPI CST 51 0% (NF 8966); NCM 33059000 IPI CST 50 14.3% (NF 8980) - conferir o cadastro do produto (IPI a menor se a alíquota correta for a maior)</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="n"/>
       <c r="F43" s="16" t="inlineStr"/>
       <c r="G43" s="16" t="inlineStr"/>
     </row>
@@ -34159,10 +34250,14 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>NF 8992/1 21/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D44" s="20" t="inlineStr"/>
+          <t>NF 786/1 02/09 YAHWEH PRINT BRASIL LTDA</t>
+        </is>
+      </c>
+      <c r="D44" s="20" t="inlineStr">
+        <is>
+          <t>VOLUMES: 4 CAIXAS</t>
+        </is>
+      </c>
       <c r="E44" s="6" t="n"/>
       <c r="F44" s="16" t="inlineStr"/>
       <c r="G44" s="16" t="inlineStr"/>
@@ -34180,14 +34275,10 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>NF 8993/1 21/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D45" s="20" t="inlineStr">
-        <is>
-          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE: 55874; INDUSTRIALIZACAO EFETUADA NA NFE 8992</t>
-        </is>
-      </c>
+          <t>NF 786/1 02/09 YAHWEH PRINT BRASIL LTDA</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="inlineStr"/>
       <c r="E45" s="6" t="n"/>
       <c r="F45" s="16" t="inlineStr"/>
       <c r="G45" s="16" t="inlineStr"/>
@@ -34205,10 +34296,14 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>NF 8993/1 21/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="inlineStr"/>
+          <t>NF 8992/1 21/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="inlineStr">
+        <is>
+          <t>INDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NAS NFs 55874 de 21-09-2026</t>
+        </is>
+      </c>
       <c r="E46" s="6" t="n"/>
       <c r="F46" s="16" t="inlineStr"/>
       <c r="G46" s="16" t="inlineStr"/>
@@ -34226,14 +34321,10 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>NF 9001/1 22/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D47" s="20" t="inlineStr">
-        <is>
-          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 55913 de 23-09-2026</t>
-        </is>
-      </c>
+          <t>NF 8992/1 21/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D47" s="20" t="inlineStr"/>
       <c r="E47" s="6" t="n"/>
       <c r="F47" s="16" t="inlineStr"/>
       <c r="G47" s="16" t="inlineStr"/>
@@ -34251,10 +34342,14 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>NF 9001/1 22/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="inlineStr"/>
+          <t>NF 8993/1 21/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="inlineStr">
+        <is>
+          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE: 55874; INDUSTRIALIZACAO EFETUADA NA NFE 8992</t>
+        </is>
+      </c>
       <c r="E48" s="6" t="n"/>
       <c r="F48" s="16" t="inlineStr"/>
       <c r="G48" s="16" t="inlineStr"/>
@@ -34272,14 +34367,10 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>NF 9002/1 22/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D49" s="20" t="inlineStr">
-        <is>
-          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 55913 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9001</t>
-        </is>
-      </c>
+          <t>NF 8993/1 21/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D49" s="20" t="inlineStr"/>
       <c r="E49" s="6" t="n"/>
       <c r="F49" s="16" t="inlineStr"/>
       <c r="G49" s="16" t="inlineStr"/>
@@ -34297,10 +34388,14 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>NF 9002/1 22/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D50" s="20" t="inlineStr"/>
+          <t>NF 9001/1 22/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="inlineStr">
+        <is>
+          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 55913 de 23-09-2026</t>
+        </is>
+      </c>
       <c r="E50" s="6" t="n"/>
       <c r="F50" s="16" t="inlineStr"/>
       <c r="G50" s="16" t="inlineStr"/>
@@ -34318,14 +34413,10 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>NF 9004/1 23/09 MIX COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D51" s="20" t="inlineStr">
-        <is>
-          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 14838 de 23-09-2026|</t>
-        </is>
-      </c>
+          <t>NF 9001/1 22/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D51" s="20" t="inlineStr"/>
       <c r="E51" s="6" t="n"/>
       <c r="F51" s="16" t="inlineStr"/>
       <c r="G51" s="16" t="inlineStr"/>
@@ -34343,10 +34434,14 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>NF 9004/1 23/09 MIX COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D52" s="20" t="inlineStr"/>
+          <t>NF 9002/1 22/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
+        <is>
+          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 55913 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9001</t>
+        </is>
+      </c>
       <c r="E52" s="6" t="n"/>
       <c r="F52" s="16" t="inlineStr"/>
       <c r="G52" s="16" t="inlineStr"/>
@@ -34364,14 +34459,10 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>NF 9005/1 23/09 MIX COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="inlineStr">
-        <is>
-          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 14838 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9004|</t>
-        </is>
-      </c>
+          <t>NF 9002/1 22/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr"/>
       <c r="E53" s="6" t="n"/>
       <c r="F53" s="16" t="inlineStr"/>
       <c r="G53" s="16" t="inlineStr"/>
@@ -34389,10 +34480,14 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>NF 9005/1 23/09 MIX COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D54" s="20" t="inlineStr"/>
+          <t>NF 9004/1 23/09 MIX COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 14838 de 23-09-2026|</t>
+        </is>
+      </c>
       <c r="E54" s="6" t="n"/>
       <c r="F54" s="16" t="inlineStr"/>
       <c r="G54" s="16" t="inlineStr"/>
@@ -34410,14 +34505,10 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>NF 9016/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="inlineStr">
-        <is>
-          <t>PESO BRUTO: 300,000</t>
-        </is>
-      </c>
+          <t>NF 9004/1 23/09 MIX COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="inlineStr"/>
       <c r="E55" s="6" t="n"/>
       <c r="F55" s="16" t="inlineStr"/>
       <c r="G55" s="16" t="inlineStr"/>
@@ -34435,10 +34526,14 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>NF 9016/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
-        </is>
-      </c>
-      <c r="D56" s="20" t="inlineStr"/>
+          <t>NF 9005/1 23/09 MIX COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 14838 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9004|</t>
+        </is>
+      </c>
       <c r="E56" s="6" t="n"/>
       <c r="F56" s="16" t="inlineStr"/>
       <c r="G56" s="16" t="inlineStr"/>
@@ -34456,14 +34551,10 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>NF 9031/1 30/09 BB COSMETICOS - EIRELI</t>
-        </is>
-      </c>
-      <c r="D57" s="20" t="inlineStr">
-        <is>
-          <t>QUANTIDADE CORRETA DE VOLUMES - 5 VOLUMES</t>
-        </is>
-      </c>
+          <t>NF 9005/1 23/09 MIX COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="inlineStr"/>
       <c r="E57" s="6" t="n"/>
       <c r="F57" s="16" t="inlineStr"/>
       <c r="G57" s="16" t="inlineStr"/>
@@ -34481,10 +34572,14 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>NF 9031/1 30/09 BB COSMETICOS - EIRELI</t>
-        </is>
-      </c>
-      <c r="D58" s="20" t="inlineStr"/>
+          <t>NF 9016/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>PESO BRUTO: 300,000</t>
+        </is>
+      </c>
       <c r="E58" s="6" t="n"/>
       <c r="F58" s="16" t="inlineStr"/>
       <c r="G58" s="16" t="inlineStr"/>
@@ -34502,14 +34597,10 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>NF 9035/1 30/09 NUTRABELLA COMERCIAL DE COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D59" s="20" t="inlineStr">
-        <is>
-          <t>Entregar:|Rua fl 9 qd 16 lt 01 casa 02, parque das flores |Cep: 74595-261|Goiania - go</t>
-        </is>
-      </c>
+          <t>NF 9016/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr"/>
       <c r="E59" s="6" t="n"/>
       <c r="F59" s="16" t="inlineStr"/>
       <c r="G59" s="16" t="inlineStr"/>
@@ -34527,10 +34618,14 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>NF 9035/1 30/09 NUTRABELLA COMERCIAL DE COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D60" s="20" t="inlineStr"/>
+          <t>NF 9031/1 30/09 BB COSMETICOS - EIRELI</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
+        <is>
+          <t>QUANTIDADE CORRETA DE VOLUMES - 5 VOLUMES</t>
+        </is>
+      </c>
       <c r="E60" s="6" t="n"/>
       <c r="F60" s="16" t="inlineStr"/>
       <c r="G60" s="16" t="inlineStr"/>
@@ -34543,19 +34638,15 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Grupo IPI</t>
+          <t>Carta de correção</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
-        </is>
-      </c>
-      <c r="D61" s="20" t="inlineStr">
-        <is>
-          <t>2 item(ns) de produto (CFOP 5124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
-        </is>
-      </c>
+          <t>NF 9031/1 30/09 BB COSMETICOS - EIRELI</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="inlineStr"/>
       <c r="E61" s="6" t="n"/>
       <c r="F61" s="16" t="inlineStr"/>
       <c r="G61" s="16" t="inlineStr"/>
@@ -34568,17 +34659,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Grupo IPI</t>
+          <t>Carta de correção</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>NF 8973/1 16/09 JORGE LEAO FERREIRA</t>
+          <t>NF 9035/1 30/09 NUTRABELLA COMERCIAL DE COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D62" s="20" t="inlineStr">
         <is>
-          <t>2 item(ns) de produto (CFOP 6124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+          <t>Entregar:|Rua fl 9 qd 16 lt 01 casa 02, parque das flores |Cep: 74595-261|Goiania - go</t>
         </is>
       </c>
       <c r="E62" s="6" t="n"/>
@@ -34593,19 +34684,15 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Grupo IPI</t>
+          <t>Carta de correção</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>NF 8980/1 17/09 GULA COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D63" s="20" t="inlineStr">
-        <is>
-          <t>3 item(ns) de produto (CFOP 5102) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
-        </is>
-      </c>
+          <t>NF 9035/1 30/09 NUTRABELLA COMERCIAL DE COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D63" s="20" t="inlineStr"/>
       <c r="E63" s="6" t="n"/>
       <c r="F63" s="16" t="inlineStr"/>
       <c r="G63" s="16" t="inlineStr"/>
@@ -34618,17 +34705,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Industrialização x retorno</t>
+          <t>Grupo IPI</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>NF 9017/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
+          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
         </is>
       </c>
       <c r="D64" s="20" t="inlineStr">
         <is>
-          <t>Informações complementares citam a industrialização na NF 9015, que é de FABIANO RODRIGUES AMARAL (CFOP 6101); a do cliente é a NF 9016 - corrigir por CC-e</t>
+          <t>2 item(ns) de produto (CFOP 5124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
         </is>
       </c>
       <c r="E64" s="6" t="n"/>
@@ -34643,17 +34730,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>NFS-e retenções</t>
+          <t>Grupo IPI</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>NFS-e 9227 01/09/2026 PLUS SANTE</t>
+          <t>NF 8973/1 16/09 JORGE LEAO FERREIRA</t>
         </is>
       </c>
       <c r="D65" s="20" t="inlineStr">
         <is>
-          <t>Serviço 0421 (atendimento médico móvel) de R$ 342.30: confirmar se há retenção de IRRF/CSRF; descontado R$ 0.00</t>
+          <t>2 item(ns) de produto (CFOP 6124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
         </is>
       </c>
       <c r="E65" s="6" t="n"/>
@@ -34668,22 +34755,20 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Remessa sem retorno</t>
+          <t>Grupo IPI</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>NF 17187 18/09 ONIXSUL COSMETICOS</t>
+          <t>NF 8980/1 17/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D66" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="n">
-        <v>5700</v>
-      </c>
+          <t>3 item(ns) de produto (CFOP 5102) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="n"/>
       <c r="F66" s="16" t="inlineStr"/>
       <c r="G66" s="16" t="inlineStr"/>
     </row>
@@ -34695,22 +34780,20 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Remessa sem retorno</t>
+          <t>Industrialização x retorno</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>NF 4551 21/09 BB COSMETICOS LTDA</t>
+          <t>NF 9017/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
         </is>
       </c>
       <c r="D67" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="n">
-        <v>65</v>
-      </c>
+          <t>Informações complementares citam a industrialização na NF 9015, que é de FABIANO RODRIGUES AMARAL (CFOP 6101); a do cliente é a NF 9016 - corrigir por CC-e</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="n"/>
       <c r="F67" s="16" t="inlineStr"/>
       <c r="G67" s="16" t="inlineStr"/>
     </row>
@@ -34722,22 +34805,20 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Remessa sem retorno</t>
+          <t>NFS-e retenções</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>NF 5027 02/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NFS-e 9227 01/09/2026 PLUS SANTE</t>
         </is>
       </c>
       <c r="D68" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE Z.R DISTRIBUIÇÃO, NF_e 4013</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="n">
-        <v>600</v>
-      </c>
+          <t>Serviço 0421 (atendimento médico móvel) de R$ 342.30: confirmar se há retenção de IRRF/CSRF; descontado R$ 0.00</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="n"/>
       <c r="F68" s="16" t="inlineStr"/>
       <c r="G68" s="16" t="inlineStr"/>
     </row>
@@ -34749,22 +34830,20 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Remessa sem retorno</t>
+          <t>PIS/COFINS no XML</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>NF 5048 03/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>35 notas 5124/6124</t>
         </is>
       </c>
       <c r="D69" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE, VITTA HAIR, OS - 166471</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="n">
-        <v>1964</v>
-      </c>
+          <t>O XML informa PIS/COFINS monofásico (CST 02, 2.2%) em R$ 115,057.65 de industrialização (PIS R$ 2,531.30 / COFINS R$ 11,850.96); a apuração usa 0,65%/3% sobre a industrialização, como nos DARFs pagos. Na encomenda de produto monofásico a alíquota concentrada é do encomendante (Lei 11.051/2004, art. 10) - corrigir o cadastro fiscal do ERP (CST 01) e confirmar o entendimento com a contadora</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="n"/>
       <c r="F69" s="16" t="inlineStr"/>
       <c r="G69" s="16" t="inlineStr"/>
     </row>
@@ -34781,16 +34860,16 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>NF 5080 09/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 17187 18/09 ONIXSUL COSMETICOS</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 165919 - ONIXSUL COSMETICOS</t>
+          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>5670</v>
+        <v>5700</v>
       </c>
       <c r="F70" s="16" t="inlineStr"/>
       <c r="G70" s="16" t="inlineStr"/>
@@ -34808,16 +34887,16 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>NF 5133 14/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 4551 21/09 BB COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D71" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 167120 - F.B. RIBEIRO E SILVA</t>
+          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>2136</v>
+        <v>65</v>
       </c>
       <c r="F71" s="16" t="inlineStr"/>
       <c r="G71" s="16" t="inlineStr"/>
@@ -34835,16 +34914,16 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>NF 5162 15/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5027 02/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D72" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE F.B RIBEIRO, OS 167134</t>
+          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE Z.R DISTRIBUIÇÃO, NF_e 4013</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>1112</v>
+        <v>600</v>
       </c>
       <c r="F72" s="16" t="inlineStr"/>
       <c r="G72" s="16" t="inlineStr"/>
@@ -34862,16 +34941,16 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>NF 5170 16/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5048 03/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D73" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE, VITTA HAIR, OS - 166471</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>667.2</v>
+        <v>1964</v>
       </c>
       <c r="F73" s="16" t="inlineStr"/>
       <c r="G73" s="16" t="inlineStr"/>
@@ -34889,16 +34968,16 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>NF 5233 21/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5080 09/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D74" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO LCIENTE, BB COSMETICOS, OS- 167541</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 165919 - ONIXSUL COSMETICOS</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>2420.01</v>
+        <v>5670</v>
       </c>
       <c r="F74" s="16" t="inlineStr"/>
       <c r="G74" s="16" t="inlineStr"/>
@@ -34916,16 +34995,16 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>NF 5235 21/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5133 14/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D75" s="20" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 166939 - Z.R. DISTRIBUIÇÃO E COMERCIO</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 167120 - F.B. RIBEIRO E SILVA</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>1760</v>
+        <v>2136</v>
       </c>
       <c r="F75" s="16" t="inlineStr"/>
       <c r="G75" s="16" t="inlineStr"/>
@@ -34943,16 +35022,16 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>NF 8099 14/09 BEPUMP IMPORTACAO E EXPORTACAO LTDA</t>
+          <t>NF 5162 15/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D76" s="20" t="inlineStr">
         <is>
-          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE F.B RIBEIRO, OS 167134</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>1408.12</v>
+        <v>1112</v>
       </c>
       <c r="F76" s="16" t="inlineStr"/>
       <c r="G76" s="16" t="inlineStr"/>
@@ -34970,23 +35049,158 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>NF 8112 14/09 OUTLET PREMIUM PACK LTDA</t>
+          <t>NF 5170 16/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D77" s="20" t="inlineStr">
         <is>
-          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>2462.03</v>
+        <v>667.2</v>
       </c>
       <c r="F77" s="16" t="inlineStr"/>
       <c r="G77" s="16" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Remessa sem retorno</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>NF 5233 21/09 JOSE DOMINGOS LINARES LTDA</t>
+        </is>
+      </c>
+      <c r="D78" s="20" t="inlineStr">
+        <is>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO LCIENTE, BB COSMETICOS, OS- 167541</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>2420.01</v>
+      </c>
+      <c r="F78" s="16" t="inlineStr"/>
+      <c r="G78" s="16" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Remessa sem retorno</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>NF 5235 21/09 JOSE DOMINGOS LINARES LTDA</t>
+        </is>
+      </c>
+      <c r="D79" s="20" t="inlineStr">
+        <is>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 166939 - Z.R. DISTRIBUIÇÃO E COMERCIO</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>1760</v>
+      </c>
+      <c r="F79" s="16" t="inlineStr"/>
+      <c r="G79" s="16" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Remessa sem retorno</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>NF 8099 14/09 BEPUMP IMPORTACAO E EXPORTACAO LTDA</t>
+        </is>
+      </c>
+      <c r="D80" s="20" t="inlineStr">
+        <is>
+          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>1408.12</v>
+      </c>
+      <c r="F80" s="16" t="inlineStr"/>
+      <c r="G80" s="16" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Remessa sem retorno</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>NF 8112 14/09 OUTLET PREMIUM PACK LTDA</t>
+        </is>
+      </c>
+      <c r="D81" s="20" t="inlineStr">
+        <is>
+          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>2462.03</v>
+      </c>
+      <c r="F81" s="16" t="inlineStr"/>
+      <c r="G81" s="16" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>XML x Registro ERP</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>30 notas de retorno 5902/6902</t>
+        </is>
+      </c>
+      <c r="D82" s="20" t="inlineStr">
+        <is>
+          <t>O Registro de Saídas do ERP não lista as notas de retorno simbólico (R$ 13,253.13); no livro/SPED elas entram (C100/C190 com CFOP 5902/6902, sem débito) - conferir no Domínio</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>13253.13</v>
+      </c>
+      <c r="F82" s="16" t="inlineStr"/>
+      <c r="G82" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Cosmetici: acumuladores do Domínio (07/08) e ICMS antecipado com saldo zero
- acumuladores de entrada por CFOP e de serviços por prestador, tirados do
  Acompanhamento de Entradas e Demonstrativo ICMS de 07 e 08/2026
- ICMS antecipado de importado lançado como débito PR000080 e crédito
  PR020212 de mesmo valor, como nos Demonstrativos (sem guia própria)
- checklist: seção L (acumuladores, 1923 e prestadores sem acumulador)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Apuracao_Fiscal_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Apuracao_Fiscal_Cosmetici_09-2026.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="B44" s="6" t="n">
-        <v>86.09</v>
+        <v>717.41</v>
       </c>
     </row>
     <row r="45">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="B47" s="6" t="n">
-        <v>-0</v>
+        <v>-631.3200000000001</v>
       </c>
     </row>
     <row r="48">
@@ -1175,202 +1175,216 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Ajuste a debito PR000080: ICMS recolhimento antecipado - importado a 4% (8% da base) - R$ 631.32 (NF 275966 MCASSAB COMERCIO E INDUSTRIA LTDA: 309.90; NF 42285 PROVITAL DO BRASIL COM. DE INSUMOS PARA COSMETICOS LTDA: 321.42)</t>
+        </is>
+      </c>
+    </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>Ajuste a credito PR020212: Crédito do ICMS antecipado (mesmo valor - saldo zero, como nos Demonstrativos 07 e 08/2026) - R$ 631.32 (NF 275966 MCASSAB COMERCIO E INDUSTRIA LTDA: 309.90; NF 42285 PROVITAL DO BRASIL COM. DE INSUMOS PARA COSMETICOS LTDA: 321.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>ICMS antecipado - entradas interestaduais a 4% (importado): 8% da base</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>NF 275966 MCASSAB COMERCIO E INDUSTRIA LTDA - TRANSCUTOL CG - TB 25 KG - base 3,873.74</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n">
+      <c r="B55" s="6" t="n">
         <v>309.9</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>NF 42285 PROVITAL DO BRASIL COM. DE INSUMOS PARA COSMETICOS LTDA - KERANUTRI - base 4,017.69</t>
         </is>
       </c>
-      <c r="B54" s="6" t="n">
+      <c r="B56" s="6" t="n">
         <v>321.42</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>Total antecipado (guia própria; no SPED: E111 PR000080 débito + PR020212 crédito, E113 por nota)</t>
-        </is>
-      </c>
-      <c r="B55" s="9" t="n">
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Total antecipado - na apuração: débito PR000080 e crédito PR020212 de mesmo valor (saldo zero, sem guia própria, como em 07 e 08/2026); E113 por nota</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="n">
         <v>631.3200000000001</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>ICMS-ST (substituto) por UF de destino</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>ICMS-ST retido - PR</t>
         </is>
       </c>
-      <c r="B58" s="6" t="n">
+      <c r="B60" s="6" t="n">
         <v>865.16</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>(-) ST de devoluções</t>
         </is>
       </c>
-      <c r="B59" s="6" t="n">
+      <c r="B61" s="6" t="n">
         <v>-0</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>ICMS-ST a recolher PR</t>
         </is>
       </c>
-      <c r="B60" s="9" t="n">
+      <c r="B62" s="9" t="n">
         <v>865.16</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>IPI</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>Débitos (saídas)</t>
         </is>
       </c>
-      <c r="B63" s="6" t="n">
+      <c r="B65" s="6" t="n">
         <v>4403.24</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>(-) Créditos (entradas)</t>
         </is>
       </c>
-      <c r="B64" s="6" t="n">
+      <c r="B66" s="6" t="n">
         <v>-2337.69</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>IPI a recolher (negativo = saldo credor)</t>
         </is>
       </c>
-      <c r="B65" s="9">
-        <f>B63+B64</f>
+      <c r="B67" s="9">
+        <f>B65+B66</f>
         <v/>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>Conferência dos documentos</t>
         </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>Notas de saída autorizadas</t>
-        </is>
-      </c>
-      <c r="B68" s="12" t="n">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>Notas canceladas (saída e entrada)</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Números inutilizados</t>
+          <t>Notas de saída autorizadas</t>
         </is>
       </c>
       <c r="B70" s="12" t="n">
-        <v>6</v>
+        <v>91</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Notas de entrada</t>
+          <t>Notas canceladas (saída e entrada)</t>
         </is>
       </c>
       <c r="B71" s="12" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>CT-e tomados</t>
+          <t>Números inutilizados</t>
         </is>
       </c>
       <c r="B72" s="12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="inlineStr">
-        <is>
-          <t>Divergências ALTA</t>
-        </is>
-      </c>
-      <c r="B73" s="14" t="n">
-        <v>9</v>
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Notas de entrada</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
+          <t>CT-e tomados</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>Divergências ALTA</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
           <t>Divergências (total)</t>
         </is>
       </c>
-      <c r="B74" s="12" t="n">
+      <c r="B76" s="12" t="n">
         <v>74</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
         <is>
           <t>Observações para a contadora</t>
         </is>
       </c>
-      <c r="B75" s="12" t="n">
+      <c r="B77" s="12" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Cosmetici: escrituração segue o XML, sem correções
- NFS-e tomadas: extrai valor, base, ISS, ISS retido, IRRF, PIS, COFINS,
  outras retenções e líquido exatamente como na nota; não recalcula
  retenção devida (removidos os alertas de retenção a menor)
- revisão das saídas e Simples: textos só informativos, sem sugerir
  CC-e, regularização ou pedido de correção ao fornecedor
- regra registrada na skill e no checklist

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Apuracao_Fiscal_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Apuracao_Fiscal_Cosmetici_09-2026.xlsx
@@ -1375,7 +1375,7 @@
         </is>
       </c>
       <c r="B76" s="12" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="77">
@@ -2230,29 +2230,29 @@
       <c r="G21" s="17" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Serviços</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
-        <is>
-          <t>NFS-e tomadas: retenção de IRRF e PIS/COFINS/CSLL</t>
-        </is>
-      </c>
-      <c r="C22" s="20" t="inlineStr">
-        <is>
-          <t>1 MÉDIA, 1 BAIXA (aba Divergências)</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>VERIFICAR</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>Lei 10.833/2003 art. 30 e 31 §3º (dispensa até R$ 10); RIR/2018 art. 714 e 716; IN SRF 459/2004</t>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>NFS-e tomadas: retenções extraídas do documento (sem recálculo)</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>21 notas extraídas (aba NFS-e tomadas)</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>Escritura-se o que consta na nota</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr"/>
@@ -33215,7 +33215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34113,7 +34113,7 @@
       </c>
       <c r="D36" s="20" t="inlineStr">
         <is>
-          <t>CFOP 5124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês. Confirmar o insumo enviado pelo encomendante; se não houve, é venda (5101/6101): PIS/COFINS monofásico 2,2%/10,3% em vez de 0,65%/3% (diferença ~R$ 39.61) e IPI tributado</t>
+          <t>CFOP 5124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês - informativo (escriturado conforme o XML, CFOP 5124)</t>
         </is>
       </c>
       <c r="E36" s="24" t="n">
@@ -34140,7 +34140,7 @@
       </c>
       <c r="D37" s="20" t="inlineStr">
         <is>
-          <t>CFOP 6124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês. Confirmar o insumo enviado pelo encomendante; se não houve, é venda (5101/6101): PIS/COFINS monofásico 2,2%/10,3% em vez de 0,65%/3% (diferença ~R$ 337.29) e IPI tributado</t>
+          <t>CFOP 6124 sem nota de remessa citada, sem retorno 5902/6902 e sem remessa recebida do cliente no mês - informativo (escriturado conforme o XML, CFOP 6124)</t>
         </is>
       </c>
       <c r="E37" s="24" t="n">
@@ -34157,47 +34157,45 @@
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>NFS-e retenções</t>
+          <t>Produto com tratamento diferente</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>NFS-e 18 01/09/2026 GENESIS ALIANCA</t>
+          <t>NEUTRALIZANTE ALL NATURE - 500ML (cód. 51)</t>
         </is>
       </c>
       <c r="D38" s="20" t="inlineStr">
         <is>
-          <t>Serviço 0401 (medicina) de R$ 728.14, prestador fora do Simples: reter IRRF 1.5% R$ 10.92 + PIS/COFINS/CSLL 4,65% R$ 33.86 = R$ 44.78; descontado na nota R$ 10.92 (diferença R$ 33.86). Conferir pagamento e DARF 1708/5952</t>
-        </is>
-      </c>
-      <c r="E38" s="24" t="n">
-        <v>33.86</v>
-      </c>
+          <t>Mesmo produto vendido no mês com NCM/IPI diferentes: NCM 33059000 IPI CST 51 0% (NF 8966); NCM 33059000 IPI CST 50 14.3% (NF 8980) - conferir o cadastro do produto (IPI a menor se a alíquota correta for a maior)</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="n"/>
       <c r="F38" s="17" t="inlineStr"/>
       <c r="G38" s="17" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>Produto com tratamento diferente</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>NEUTRALIZANTE ALL NATURE - 500ML (cód. 51)</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="inlineStr">
-        <is>
-          <t>Mesmo produto vendido no mês com NCM/IPI diferentes: NCM 33059000 IPI CST 51 0% (NF 8966); NCM 33059000 IPI CST 50 14.3% (NF 8980) - conferir o cadastro do produto (IPI a menor se a alíquota correta for a maior)</t>
-        </is>
-      </c>
-      <c r="E39" s="24" t="n"/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Carta de correção</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>NF 786/1 02/09 YAHWEH PRINT BRASIL LTDA</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>VOLUMES: 4 CAIXAS</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n"/>
       <c r="F39" s="17" t="inlineStr"/>
       <c r="G39" s="17" t="inlineStr"/>
     </row>
@@ -34217,11 +34215,7 @@
           <t>NF 786/1 02/09 YAHWEH PRINT BRASIL LTDA</t>
         </is>
       </c>
-      <c r="D40" s="21" t="inlineStr">
-        <is>
-          <t>VOLUMES: 4 CAIXAS</t>
-        </is>
-      </c>
+      <c r="D40" s="21" t="inlineStr"/>
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="17" t="inlineStr"/>
       <c r="G40" s="17" t="inlineStr"/>
@@ -34239,10 +34233,14 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>NF 786/1 02/09 YAHWEH PRINT BRASIL LTDA</t>
-        </is>
-      </c>
-      <c r="D41" s="21" t="inlineStr"/>
+          <t>NF 8992/1 21/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D41" s="21" t="inlineStr">
+        <is>
+          <t>INDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NAS NFs 55874 de 21-09-2026</t>
+        </is>
+      </c>
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="17" t="inlineStr"/>
       <c r="G41" s="17" t="inlineStr"/>
@@ -34263,11 +34261,7 @@
           <t>NF 8992/1 21/09 MIX PERFUMARIA LTDA</t>
         </is>
       </c>
-      <c r="D42" s="21" t="inlineStr">
-        <is>
-          <t>INDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NAS NFs 55874 de 21-09-2026</t>
-        </is>
-      </c>
+      <c r="D42" s="21" t="inlineStr"/>
       <c r="E42" s="6" t="n"/>
       <c r="F42" s="17" t="inlineStr"/>
       <c r="G42" s="17" t="inlineStr"/>
@@ -34285,10 +34279,14 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>NF 8992/1 21/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D43" s="21" t="inlineStr"/>
+          <t>NF 8993/1 21/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D43" s="21" t="inlineStr">
+        <is>
+          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE: 55874; INDUSTRIALIZACAO EFETUADA NA NFE 8992</t>
+        </is>
+      </c>
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="17" t="inlineStr"/>
       <c r="G43" s="17" t="inlineStr"/>
@@ -34309,11 +34307,7 @@
           <t>NF 8993/1 21/09 MIX PERFUMARIA LTDA</t>
         </is>
       </c>
-      <c r="D44" s="21" t="inlineStr">
-        <is>
-          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE: 55874; INDUSTRIALIZACAO EFETUADA NA NFE 8992</t>
-        </is>
-      </c>
+      <c r="D44" s="21" t="inlineStr"/>
       <c r="E44" s="6" t="n"/>
       <c r="F44" s="17" t="inlineStr"/>
       <c r="G44" s="17" t="inlineStr"/>
@@ -34331,10 +34325,14 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>NF 8993/1 21/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D45" s="21" t="inlineStr"/>
+          <t>NF 9001/1 22/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D45" s="21" t="inlineStr">
+        <is>
+          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 55913 de 23-09-2026</t>
+        </is>
+      </c>
       <c r="E45" s="6" t="n"/>
       <c r="F45" s="17" t="inlineStr"/>
       <c r="G45" s="17" t="inlineStr"/>
@@ -34355,11 +34353,7 @@
           <t>NF 9001/1 22/09 MIX PERFUMARIA LTDA</t>
         </is>
       </c>
-      <c r="D46" s="21" t="inlineStr">
-        <is>
-          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 55913 de 23-09-2026</t>
-        </is>
-      </c>
+      <c r="D46" s="21" t="inlineStr"/>
       <c r="E46" s="6" t="n"/>
       <c r="F46" s="17" t="inlineStr"/>
       <c r="G46" s="17" t="inlineStr"/>
@@ -34377,10 +34371,14 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>NF 9001/1 22/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D47" s="21" t="inlineStr"/>
+          <t>NF 9002/1 22/09 MIX PERFUMARIA LTDA</t>
+        </is>
+      </c>
+      <c r="D47" s="21" t="inlineStr">
+        <is>
+          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 55913 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9001</t>
+        </is>
+      </c>
       <c r="E47" s="6" t="n"/>
       <c r="F47" s="17" t="inlineStr"/>
       <c r="G47" s="17" t="inlineStr"/>
@@ -34401,11 +34399,7 @@
           <t>NF 9002/1 22/09 MIX PERFUMARIA LTDA</t>
         </is>
       </c>
-      <c r="D48" s="21" t="inlineStr">
-        <is>
-          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 55913 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9001</t>
-        </is>
-      </c>
+      <c r="D48" s="21" t="inlineStr"/>
       <c r="E48" s="6" t="n"/>
       <c r="F48" s="17" t="inlineStr"/>
       <c r="G48" s="17" t="inlineStr"/>
@@ -34423,10 +34417,14 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>NF 9002/1 22/09 MIX PERFUMARIA LTDA</t>
-        </is>
-      </c>
-      <c r="D49" s="21" t="inlineStr"/>
+          <t>NF 9004/1 23/09 MIX COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D49" s="21" t="inlineStr">
+        <is>
+          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 14838 de 23-09-2026|</t>
+        </is>
+      </c>
       <c r="E49" s="6" t="n"/>
       <c r="F49" s="17" t="inlineStr"/>
       <c r="G49" s="17" t="inlineStr"/>
@@ -34447,11 +34445,7 @@
           <t>NF 9004/1 23/09 MIX COSMETICOS LTDA</t>
         </is>
       </c>
-      <c r="D50" s="21" t="inlineStr">
-        <is>
-          <t>INSDUSTRIALIZACAO EFETUADA COM INSUMOS ENVIADOS NA NFE 14838 de 23-09-2026|</t>
-        </is>
-      </c>
+      <c r="D50" s="21" t="inlineStr"/>
       <c r="E50" s="6" t="n"/>
       <c r="F50" s="17" t="inlineStr"/>
       <c r="G50" s="17" t="inlineStr"/>
@@ -34469,10 +34463,14 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>NF 9004/1 23/09 MIX COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D51" s="21" t="inlineStr"/>
+          <t>NF 9005/1 23/09 MIX COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 14838 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9004|</t>
+        </is>
+      </c>
       <c r="E51" s="6" t="n"/>
       <c r="F51" s="17" t="inlineStr"/>
       <c r="G51" s="17" t="inlineStr"/>
@@ -34493,11 +34491,7 @@
           <t>NF 9005/1 23/09 MIX COSMETICOS LTDA</t>
         </is>
       </c>
-      <c r="D52" s="21" t="inlineStr">
-        <is>
-          <t>RETORNO SIMBOLICO DOS INSUMOS ENVIADOS NA NFE 14838 DE 23-09-26 ; INDUSTRIALIZACAO EFETUADA NA NFE 9004|</t>
-        </is>
-      </c>
+      <c r="D52" s="21" t="inlineStr"/>
       <c r="E52" s="6" t="n"/>
       <c r="F52" s="17" t="inlineStr"/>
       <c r="G52" s="17" t="inlineStr"/>
@@ -34515,10 +34509,14 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>NF 9005/1 23/09 MIX COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D53" s="21" t="inlineStr"/>
+          <t>NF 9016/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>PESO BRUTO: 300,000</t>
+        </is>
+      </c>
       <c r="E53" s="6" t="n"/>
       <c r="F53" s="17" t="inlineStr"/>
       <c r="G53" s="17" t="inlineStr"/>
@@ -34539,11 +34537,7 @@
           <t>NF 9016/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
         </is>
       </c>
-      <c r="D54" s="21" t="inlineStr">
-        <is>
-          <t>PESO BRUTO: 300,000</t>
-        </is>
-      </c>
+      <c r="D54" s="21" t="inlineStr"/>
       <c r="E54" s="6" t="n"/>
       <c r="F54" s="17" t="inlineStr"/>
       <c r="G54" s="17" t="inlineStr"/>
@@ -34561,10 +34555,14 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>NF 9016/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="inlineStr"/>
+          <t>NF 9031/1 30/09 BB COSMETICOS - EIRELI</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
+        <is>
+          <t>QUANTIDADE CORRETA DE VOLUMES - 5 VOLUMES</t>
+        </is>
+      </c>
       <c r="E55" s="6" t="n"/>
       <c r="F55" s="17" t="inlineStr"/>
       <c r="G55" s="17" t="inlineStr"/>
@@ -34585,11 +34583,7 @@
           <t>NF 9031/1 30/09 BB COSMETICOS - EIRELI</t>
         </is>
       </c>
-      <c r="D56" s="21" t="inlineStr">
-        <is>
-          <t>QUANTIDADE CORRETA DE VOLUMES - 5 VOLUMES</t>
-        </is>
-      </c>
+      <c r="D56" s="21" t="inlineStr"/>
       <c r="E56" s="6" t="n"/>
       <c r="F56" s="17" t="inlineStr"/>
       <c r="G56" s="17" t="inlineStr"/>
@@ -34607,10 +34601,14 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>NF 9031/1 30/09 BB COSMETICOS - EIRELI</t>
-        </is>
-      </c>
-      <c r="D57" s="21" t="inlineStr"/>
+          <t>NF 9035/1 30/09 NUTRABELLA COMERCIAL DE COSMETICOS LTDA</t>
+        </is>
+      </c>
+      <c r="D57" s="21" t="inlineStr">
+        <is>
+          <t>Entregar:|Rua fl 9 qd 16 lt 01 casa 02, parque das flores |Cep: 74595-261|Goiania - go</t>
+        </is>
+      </c>
       <c r="E57" s="6" t="n"/>
       <c r="F57" s="17" t="inlineStr"/>
       <c r="G57" s="17" t="inlineStr"/>
@@ -34631,11 +34629,7 @@
           <t>NF 9035/1 30/09 NUTRABELLA COMERCIAL DE COSMETICOS LTDA</t>
         </is>
       </c>
-      <c r="D58" s="21" t="inlineStr">
-        <is>
-          <t>Entregar:|Rua fl 9 qd 16 lt 01 casa 02, parque das flores |Cep: 74595-261|Goiania - go</t>
-        </is>
-      </c>
+      <c r="D58" s="21" t="inlineStr"/>
       <c r="E58" s="6" t="n"/>
       <c r="F58" s="17" t="inlineStr"/>
       <c r="G58" s="17" t="inlineStr"/>
@@ -34648,15 +34642,19 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Carta de correção</t>
+          <t>Grupo IPI</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>NF 9035/1 30/09 NUTRABELLA COMERCIAL DE COSMETICOS LTDA</t>
-        </is>
-      </c>
-      <c r="D59" s="21" t="inlineStr"/>
+          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
+        </is>
+      </c>
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>2 item(ns) de produto (CFOP 5124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+        </is>
+      </c>
       <c r="E59" s="6" t="n"/>
       <c r="F59" s="17" t="inlineStr"/>
       <c r="G59" s="17" t="inlineStr"/>
@@ -34674,12 +34672,12 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>NF 8939/1 02/09 CANDIDO COMERCIO DE COSMETICOS - EIRELI</t>
+          <t>NF 8973/1 16/09 JORGE LEAO FERREIRA</t>
         </is>
       </c>
       <c r="D60" s="21" t="inlineStr">
         <is>
-          <t>2 item(ns) de produto (CFOP 5124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+          <t>2 item(ns) de produto (CFOP 6124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
         </is>
       </c>
       <c r="E60" s="6" t="n"/>
@@ -34699,12 +34697,12 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>NF 8973/1 16/09 JORGE LEAO FERREIRA</t>
+          <t>NF 8980/1 17/09 GULA COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D61" s="21" t="inlineStr">
         <is>
-          <t>2 item(ns) de produto (CFOP 6124) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+          <t>3 item(ns) de produto (CFOP 5102) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
         </is>
       </c>
       <c r="E61" s="6" t="n"/>
@@ -34719,17 +34717,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Grupo IPI</t>
+          <t>Industrialização x retorno</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>NF 8980/1 17/09 GULA COSMETICOS LTDA</t>
+          <t>NF 9017/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
         <is>
-          <t>3 item(ns) de produto (CFOP 5102) sem grupo de IPI (CST) - conferir o cadastro do produto no ERP</t>
+          <t>Informações complementares citam a industrialização na NF 9015, que é de FABIANO RODRIGUES AMARAL (CFOP 6101); a do cliente é a NF 9016 - informativo, escriturado como está no XML</t>
         </is>
       </c>
       <c r="E62" s="6" t="n"/>
@@ -34744,17 +34742,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Industrialização x retorno</t>
+          <t>PIS/COFINS no XML</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>NF 9017/1 28/09 LUAN PATRICK LORANDI 02301366057</t>
+          <t>35 notas 5124/6124</t>
         </is>
       </c>
       <c r="D63" s="21" t="inlineStr">
         <is>
-          <t>Informações complementares citam a industrialização na NF 9015, que é de FABIANO RODRIGUES AMARAL (CFOP 6101); a do cliente é a NF 9016 - corrigir por CC-e</t>
+          <t>O XML informa PIS/COFINS monofásico (CST 02, 2.2%) em R$ 115,057.65 de industrialização (PIS R$ 2,531.30 / COFINS R$ 11,850.96); a apuração usa 0,65%/3% sobre a industrialização, como nos DARFs pagos. Na encomenda de produto monofásico a alíquota concentrada é do encomendante (Lei 11.051/2004, art. 10) - informativo - a nota é escriturada como emitida</t>
         </is>
       </c>
       <c r="E63" s="6" t="n"/>
@@ -34769,20 +34767,22 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>NFS-e retenções</t>
+          <t>Remessa sem retorno</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>NFS-e 9227 01/09/2026 PLUS SANTE</t>
+          <t>NF 17187 18/09 ONIXSUL COSMETICOS</t>
         </is>
       </c>
       <c r="D64" s="21" t="inlineStr">
         <is>
-          <t>Serviço 0421 (atendimento médico móvel) de R$ 342.30: confirmar se há retenção de IRRF/CSRF; descontado R$ 0.00</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="n"/>
+          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="n">
+        <v>5700</v>
+      </c>
       <c r="F64" s="17" t="inlineStr"/>
       <c r="G64" s="17" t="inlineStr"/>
     </row>
@@ -34794,20 +34794,22 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>PIS/COFINS no XML</t>
+          <t>Remessa sem retorno</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>35 notas 5124/6124</t>
+          <t>NF 4551 21/09 BB COSMETICOS LTDA</t>
         </is>
       </c>
       <c r="D65" s="21" t="inlineStr">
         <is>
-          <t>O XML informa PIS/COFINS monofásico (CST 02, 2.2%) em R$ 115,057.65 de industrialização (PIS R$ 2,531.30 / COFINS R$ 11,850.96); a apuração usa 0,65%/3% sobre a industrialização, como nos DARFs pagos. Na encomenda de produto monofásico a alíquota concentrada é do encomendante (Lei 11.051/2004, art. 10) - corrigir o cadastro fiscal do ERP (CST 01) e confirmar o entendimento com a contadora</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="n"/>
+          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>65</v>
+      </c>
       <c r="F65" s="17" t="inlineStr"/>
       <c r="G65" s="17" t="inlineStr"/>
     </row>
@@ -34824,16 +34826,16 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>NF 17187 18/09 ONIXSUL COSMETICOS</t>
+          <t>NF 5027 02/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D66" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE Z.R DISTRIBUIÇÃO, NF_e 4013</t>
         </is>
       </c>
       <c r="E66" s="6" t="n">
-        <v>5700</v>
+        <v>600</v>
       </c>
       <c r="F66" s="17" t="inlineStr"/>
       <c r="G66" s="17" t="inlineStr"/>
@@ -34851,16 +34853,16 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>NF 4551 21/09 BB COSMETICOS LTDA</t>
+          <t>NF 5048 03/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D67" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5901 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE, VITTA HAIR, OS - 166471</t>
         </is>
       </c>
       <c r="E67" s="6" t="n">
-        <v>65</v>
+        <v>1964</v>
       </c>
       <c r="F67" s="17" t="inlineStr"/>
       <c r="G67" s="17" t="inlineStr"/>
@@ -34878,16 +34880,16 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>NF 5027 02/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5080 09/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE Z.R DISTRIBUIÇÃO, NF_e 4013</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 165919 - ONIXSUL COSMETICOS</t>
         </is>
       </c>
       <c r="E68" s="6" t="n">
-        <v>600</v>
+        <v>5670</v>
       </c>
       <c r="F68" s="17" t="inlineStr"/>
       <c r="G68" s="17" t="inlineStr"/>
@@ -34905,16 +34907,16 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>NF 5048 03/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5133 14/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D69" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE, VITTA HAIR, OS - 166471</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 167120 - F.B. RIBEIRO E SILVA</t>
         </is>
       </c>
       <c r="E69" s="6" t="n">
-        <v>1964</v>
+        <v>2136</v>
       </c>
       <c r="F69" s="17" t="inlineStr"/>
       <c r="G69" s="17" t="inlineStr"/>
@@ -34932,16 +34934,16 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>NF 5080 09/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5162 15/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D70" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 165919 - ONIXSUL COSMETICOS</t>
+          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE F.B RIBEIRO, OS 167134</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>5670</v>
+        <v>1112</v>
       </c>
       <c r="F70" s="17" t="inlineStr"/>
       <c r="G70" s="17" t="inlineStr"/>
@@ -34959,16 +34961,16 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>NF 5133 14/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5170 16/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D71" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 167120 - F.B. RIBEIRO E SILVA</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>2136</v>
+        <v>667.2</v>
       </c>
       <c r="F71" s="17" t="inlineStr"/>
       <c r="G71" s="17" t="inlineStr"/>
@@ -34986,16 +34988,16 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>NF 5162 15/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5233 21/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D72" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5923 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO CLIENTE F.B RIBEIRO, OS 167134</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO LCIENTE, BB COSMETICOS, OS- 167541</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>1112</v>
+        <v>2420.01</v>
       </c>
       <c r="F72" s="17" t="inlineStr"/>
       <c r="G72" s="17" t="inlineStr"/>
@@ -35013,16 +35015,16 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>NF 5170 16/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 5235 21/09 JOSE DOMINGOS LINARES LTDA</t>
         </is>
       </c>
       <c r="D73" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 166939 - Z.R. DISTRIBUIÇÃO E COMERCIO</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>667.2</v>
+        <v>1760</v>
       </c>
       <c r="F73" s="17" t="inlineStr"/>
       <c r="G73" s="17" t="inlineStr"/>
@@ -35040,16 +35042,16 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>NF 5233 21/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 8099 14/09 BEPUMP IMPORTACAO E EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="D74" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE AO LCIENTE, BB COSMETICOS, OS- 167541</t>
+          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>2420.01</v>
+        <v>1408.12</v>
       </c>
       <c r="F74" s="17" t="inlineStr"/>
       <c r="G74" s="17" t="inlineStr"/>
@@ -35067,16 +35069,16 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>NF 5235 21/09 JOSE DOMINGOS LINARES LTDA</t>
+          <t>NF 8112 14/09 OUTLET PREMIUM PACK LTDA</t>
         </is>
       </c>
       <c r="D75" s="21" t="inlineStr">
         <is>
-          <t>Remessa 5924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle). REFERENTE A OS 166939 - Z.R. DISTRIBUIÇÃO E COMERCIO</t>
+          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>1760</v>
+        <v>2462.03</v>
       </c>
       <c r="F75" s="17" t="inlineStr"/>
       <c r="G75" s="17" t="inlineStr"/>
@@ -35089,82 +35091,28 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Remessa sem retorno</t>
+          <t>XML x Registro ERP</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>NF 8099 14/09 BEPUMP IMPORTACAO E EXPORTACAO LTDA</t>
+          <t>30 notas de retorno 5902/6902</t>
         </is>
       </c>
       <c r="D76" s="21" t="inlineStr">
         <is>
-          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
+          <t>O Registro de Saídas do ERP não lista as notas de retorno simbólico (R$ 13,253.13); no livro/SPED elas entram (C100/C190 com CFOP 5902/6902, sem débito) - conferir no Domínio</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>1408.12</v>
+        <v>13253.13</v>
       </c>
       <c r="F76" s="17" t="inlineStr"/>
       <c r="G76" s="17" t="inlineStr"/>
     </row>
-    <row r="77">
-      <c r="A77" s="5" t="inlineStr">
-        <is>
-          <t>BAIXA</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>Remessa sem retorno</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>NF 8112 14/09 OUTLET PREMIUM PACK LTDA</t>
-        </is>
-      </c>
-      <c r="D77" s="21" t="inlineStr">
-        <is>
-          <t>Remessa 6924 recebida e ainda sem retorno citado no mês - fica no estoque de terceiros (controle)</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="n">
-        <v>2462.03</v>
-      </c>
-      <c r="F77" s="17" t="inlineStr"/>
-      <c r="G77" s="17" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>BAIXA</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>XML x Registro ERP</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>30 notas de retorno 5902/6902</t>
-        </is>
-      </c>
-      <c r="D78" s="21" t="inlineStr">
-        <is>
-          <t>O Registro de Saídas do ERP não lista as notas de retorno simbólico (R$ 13,253.13); no livro/SPED elas entram (C100/C190 com CFOP 5902/6902, sem débito) - conferir no Domínio</t>
-        </is>
-      </c>
-      <c r="E78" s="6" t="n">
-        <v>13253.13</v>
-      </c>
-      <c r="F78" s="17" t="inlineStr"/>
-      <c r="G78" s="17" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -35198,10 +35146,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="45" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>2. Insumo de cliente emitido com CFOP 5124/6124 soma R$ 3,004.50 (aba Divergências, "Industrialização x retorno"). Está na base do PIS/COFINS (0,65%/3% = R$ 19.53 + R$ 90.13) e do IRPJ/CSLL. Se a contadora confirmar que é retorno em duplicidade, tirar da base e pedir ao cliente a regularização (CC-e do CFOP não altera valores - Ajuste SINIEF 01/07; senão, nota de entrada/anulação conforme RICMS/PR).</t>
+          <t>2. Insumo de cliente emitido com CFOP 5124/6124 soma R$ 3,004.50 (aba Divergências, "Industrialização x retorno"). Está na base do PIS/COFINS (0,65%/3% = R$ 19.53 + R$ 90.13) e do IRPJ/CSLL. Informativo: a escrituração segue o XML (nada é alterado).</t>
         </is>
       </c>
     </row>

</xml_diff>